<commit_message>
generated 10 of 20 production modules
</commit_message>
<xml_diff>
--- a/iBag597-BiGG.xlsx
+++ b/iBag597-BiGG.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/matthewchung/utk/iBag/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4FD512B-E0C7-824B-8817-7D0D4837937A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F42A3BA3-2D55-AB49-ACF7-E30E788E9CB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="440" yWindow="1140" windowWidth="27640" windowHeight="16660" xr2:uid="{CED1CA87-81C3-A440-8918-3F231FDC256A}"/>
   </bookViews>
@@ -2467,29 +2467,33 @@
       <c r="E60" s="4"/>
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="B62" s="6"/>
+      <c r="A62" s="6"/>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A63" s="6"/>
       <c r="C63" s="4"/>
       <c r="D63" s="4"/>
       <c r="E63" s="4"/>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A64" s="6"/>
       <c r="B64" s="6"/>
       <c r="C64" s="5"/>
       <c r="D64" s="6"/>
     </row>
-    <row r="65" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A65" s="6"/>
       <c r="C65" s="5"/>
     </row>
-    <row r="66" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A66" s="6"/>
       <c r="C66" s="5"/>
       <c r="E66" s="7"/>
     </row>
-    <row r="67" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:5" x14ac:dyDescent="0.35">
       <c r="E67" s="4"/>
     </row>
-    <row r="68" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B68" s="7"/>
       <c r="E68" s="4"/>
     </row>

</xml_diff>